<commit_message>
data: update 데이터변경이력.xlsx for 2026-08-28
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/데이터변경이력.xlsx
+++ b/docs/dashboard/data/데이터변경이력.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:J167"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="20.0" customWidth="true"/>
@@ -168,7 +168,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 16:08:59</t>
+          <t>2026-08-27 15:25:47</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -193,34 +193,34 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>등록</t>
+          <t>수정</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>CM-TL-0224 Optical Power Meter</t>
+          <t>CM-TL-0223 Optiocal Laser Source</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>모델</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>LOS-36V2</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>OLS-36V2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 16:07:31</t>
+          <t>2026-08-26 16:08:59</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -250,7 +250,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>CM-TL-0223 Optiocal Laser Source</t>
+          <t>CM-TL-0224 Optical Power Meter</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -272,27 +272,27 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 08:11:42</t>
+          <t>2026-08-26 16:07:31</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>주식회사 카프마이크로</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>최문정</t>
+          <t>김호영</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>mjchoi@shinhwa-pritech.com</t>
+          <t>hoykim@caphmicro.com</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>사용자 관리</t>
+          <t>계측기 통합 대장</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -302,7 +302,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>김혜민</t>
+          <t>CM-TL-0223 Optiocal Laser Source</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -317,66 +317,66 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>사용자 등록</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 09:56:13</t>
+          <t>2026-08-21 08:11:42</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아(주)</t>
+          <t>(주)신화프리텍</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>전승헌</t>
+          <t>최문정</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>sh.chun@avjet.kr</t>
+          <t>mjchoi@shinhwa-pritech.com</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>계측기 통합 대장</t>
+          <t>사용자 관리</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>수정</t>
+          <t>등록</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>125 KIT STRUT SERVICE</t>
+          <t>김혜민</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>설치 위치</t>
+          <t/>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>FIC</t>
+          <t/>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>FIC &gt; 1호기 &gt; 장비실 &gt; J3</t>
+          <t>사용자 등록</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 09:50:47</t>
+          <t>2026-08-19 09:56:13</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -416,19 +416,19 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>FIC</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>FIC &gt; 1호기 &gt; 장비실 &gt; J3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 09:45:48</t>
+          <t>2026-08-19 09:50:47</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -453,7 +453,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>등록</t>
+          <t>수정</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -463,7 +463,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>설치 위치</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -473,34 +473,34 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>J3</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:48:49</t>
+          <t>2026-08-19 09:45:48</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>주식회사 카프마이크로</t>
+          <t>에브제트아시아(주)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>박준영</t>
+          <t>전승헌</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>jypark@caphmicro.com</t>
+          <t>sh.chun@avjet.kr</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>사용자 관리</t>
+          <t>계측기 통합 대장</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>김호영</t>
+          <t>125 KIT STRUT SERVICE</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -525,14 +525,14 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>사용자 등록</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:35:09</t>
+          <t>2026-08-18 11:48:49</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -552,39 +552,39 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>계측기 통합 대장</t>
+          <t>사용자 관리</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>수정</t>
+          <t>등록</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>CM-0047 디지털 게이지</t>
+          <t>김호영</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>모델</t>
+          <t/>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>33574</t>
+          <t/>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>ID-C1012</t>
+          <t>사용자 등록</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:13:35</t>
+          <t>2026-08-18 11:35:09</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -614,29 +614,29 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>CM-0060 Digital Push Pull Gage</t>
+          <t>CM-0047 디지털 게이지</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>상태</t>
+          <t>모델</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>정상</t>
+          <t>33574</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>미사용</t>
+          <t>ID-C1012</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:13:28</t>
+          <t>2026-08-18 11:13:35</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>CM-0059 Digital Push Pull Gage</t>
+          <t>CM-0060 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:13:21</t>
+          <t>2026-08-18 11:13:28</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>CM-0058 Digital Push Pull Gage</t>
+          <t>CM-0059 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -740,7 +740,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:13:11</t>
+          <t>2026-08-18 11:13:21</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>CM-0056 인두팁 온도계</t>
+          <t>CM-0058 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -792,7 +792,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:13:03</t>
+          <t>2026-08-18 11:13:11</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>CM-0055 디지털테스터</t>
+          <t>CM-0056 인두팁 온도계</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:12:54</t>
+          <t>2026-08-18 11:13:03</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>CM-0053 전자기 방사선 측정기</t>
+          <t>CM-0055 디지털테스터</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:12:47</t>
+          <t>2026-08-18 11:12:54</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>CM-0052 Cable Tester and Digital Multimeter</t>
+          <t>CM-0053 전자기 방사선 측정기</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:12:39</t>
+          <t>2026-08-18 11:12:47</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>CM-0051 휴대용 소음 감지기</t>
+          <t>CM-0052 Cable Tester and Digital Multimeter</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1000,7 +1000,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:12:31</t>
+          <t>2026-08-18 11:12:39</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>CM-0050 Digital Push Pull Gage</t>
+          <t>CM-0051 휴대용 소음 감지기</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1052,7 +1052,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:12:23</t>
+          <t>2026-08-18 11:12:31</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>CM-0049 버니어켈리퍼스</t>
+          <t>CM-0050 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1104,7 +1104,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:12:16</t>
+          <t>2026-08-18 11:12:23</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>CM-0048 디지털 토크 드라이버 셋트</t>
+          <t>CM-0049 버니어켈리퍼스</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1156,7 +1156,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:12:09</t>
+          <t>2026-08-18 11:12:16</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>CM-0047 디지털 게이지</t>
+          <t>CM-0048 디지털 토크 드라이버 셋트</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1208,7 +1208,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:12:01</t>
+          <t>2026-08-18 11:12:09</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>CM-0046 Milliohm Meter</t>
+          <t>CM-0047 디지털 게이지</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1260,7 +1260,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:11:53</t>
+          <t>2026-08-18 11:12:01</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>CM-0045 전자저울</t>
+          <t>CM-0046 Milliohm Meter</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1312,7 +1312,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:11:44</t>
+          <t>2026-08-18 11:11:53</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>CM-0044 Force Gauge</t>
+          <t>CM-0045 전자저울</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1364,7 +1364,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:11:17</t>
+          <t>2026-08-18 11:11:44</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>CM-0043 Digital Push Pull Gage</t>
+          <t>CM-0044 Force Gauge</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:11:06</t>
+          <t>2026-08-18 11:11:17</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>CM-0033 CABLE&amp;HARNESS MULTI TESTER</t>
+          <t>CM-0043 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:10:44</t>
+          <t>2026-08-18 11:11:06</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>CM-0022 광 측정기</t>
+          <t>CM-0033 CABLE&amp;HARNESS MULTI TESTER</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:10:25</t>
+          <t>2026-08-18 11:10:44</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>CM-0042 HiTESTER</t>
+          <t>CM-0022 광 측정기</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:09:52</t>
+          <t>2026-08-18 11:10:25</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1597,34 +1597,34 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>등록</t>
+          <t>수정</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>CM-0060 Digital Push Pull Gage</t>
+          <t>CM-0042 HiTESTER</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>상태</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>정상</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>미사용</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:09:03</t>
+          <t>2026-08-18 11:09:52</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>CM-0059 Digital Push Pull Gage</t>
+          <t>CM-0060 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1676,7 +1676,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:08:31</t>
+          <t>2026-08-18 11:09:03</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>CM-0058 Digital Push Pull Gage</t>
+          <t>CM-0059 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1728,7 +1728,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 11:07:55</t>
+          <t>2026-08-18 11:08:31</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>CM-0057 버니어켈리퍼스</t>
+          <t>CM-0058 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>CM-0057_내외측 켈리퍼(Digamatic Calipers)_251203_대전연구소(25016231-1)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -1877,14 +1877,14 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>CM-0057_내외측 켈리퍼(Digamatic Calipers)_251203_대전연구소(25016231-1).pdf</t>
+          <t>CM-0057_내외측 켈리퍼(Digamatic Calipers)_251203_대전연구소(25016231-1)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:59:48</t>
+          <t>2026-08-18 11:07:55</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>CM-0056 인두팁 온도계</t>
+          <t>CM-0057 버니어켈리퍼스</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -1929,14 +1929,14 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0057_내외측 켈리퍼(Digamatic Calipers)_251203_대전연구소(25016231-1).pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:58:52</t>
+          <t>2026-08-18 10:59:48</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>CM-0055 디지털테스터</t>
+          <t>CM-0056 인두팁 온도계</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1988,7 +1988,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:58:01</t>
+          <t>2026-08-18 10:58:52</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>CM-0054 토크 드라이버</t>
+          <t>CM-0055 디지털테스터</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0054 260306 - 토크드라이버(457749Q)_연구개발_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -2137,14 +2137,14 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0054 260306 - 토크드라이버(457749Q)_연구개발.pdf</t>
+          <t>관리번호 CM-0054 260306 - 토크드라이버(457749Q)_연구개발_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:57:01</t>
+          <t>2026-08-18 10:58:01</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>CM-0053 전자기 방사선 측정기</t>
+          <t>CM-0054 토크 드라이버</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2189,14 +2189,14 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0054 260306 - 토크드라이버(457749Q)_연구개발.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:56:19</t>
+          <t>2026-08-18 10:57:01</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>CM-0052 Cable Tester and Digital Multimeter</t>
+          <t>CM-0053 전자기 방사선 측정기</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2248,7 +2248,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:55:45</t>
+          <t>2026-08-18 10:56:19</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>CM-0051 휴대용 소음 감지기</t>
+          <t>CM-0052 Cable Tester and Digital Multimeter</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2300,7 +2300,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:33:45</t>
+          <t>2026-08-18 10:55:45</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>CM-0050 Digital Push Pull Gage</t>
+          <t>CM-0051 휴대용 소음 감지기</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2352,7 +2352,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:33:14</t>
+          <t>2026-08-18 10:33:45</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>CM-0049 버니어켈리퍼스</t>
+          <t>CM-0050 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2404,7 +2404,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:31:52</t>
+          <t>2026-08-18 10:33:14</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>CM-0048 디지털 토크 드라이버 셋트</t>
+          <t>CM-0049 버니어켈리퍼스</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2456,7 +2456,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:31:23</t>
+          <t>2026-08-18 10:31:52</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>CM-0047 디지털 게이지</t>
+          <t>CM-0048 디지털 토크 드라이버 셋트</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2508,7 +2508,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:30:41</t>
+          <t>2026-08-18 10:31:23</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>CM-0046 Milliohm Meter</t>
+          <t>CM-0047 디지털 게이지</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2560,7 +2560,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:30:03</t>
+          <t>2026-08-18 10:30:41</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>CM-0045 전자저울</t>
+          <t>CM-0046 Milliohm Meter</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2612,7 +2612,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:29:18</t>
+          <t>2026-08-18 10:30:03</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2637,17 +2637,17 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>수정</t>
+          <t>등록</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>CM-0044 Force Gauge</t>
+          <t>CM-0045 전자저울</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>설치 위치</t>
+          <t/>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -2657,14 +2657,14 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>유휴장비보관함</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:29:10</t>
+          <t>2026-08-18 10:29:18</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>CM-0043 Digital Push Pull Gage</t>
+          <t>CM-0044 Force Gauge</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2716,7 +2716,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:28:52</t>
+          <t>2026-08-18 10:29:10</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2741,17 +2741,17 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>등록</t>
+          <t>수정</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>CM-0044 Force Gauge</t>
+          <t>CM-0043 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>설치 위치</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -2761,14 +2761,14 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>유휴장비보관함</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:28:12</t>
+          <t>2026-08-18 10:28:52</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>CM-0043 Digital Push Pull Gage</t>
+          <t>CM-0044 Force Gauge</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2820,7 +2820,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:27:42</t>
+          <t>2026-08-18 10:28:12</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>CM-0042 HiTESTER</t>
+          <t>CM-0043 Digital Push Pull Gage</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2872,7 +2872,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:26:49</t>
+          <t>2026-08-18 10:27:42</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>CM-0041 토크 드라이버</t>
+          <t>CM-0042 HiTESTER</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0041 260306 - 토크드라이버(CM-E-0033)_연구개발_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -3021,14 +3021,14 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0041 260306 - 토크드라이버(CM-E-0033)_연구개발.pdf</t>
+          <t>관리번호 CM-0041 260306 - 토크드라이버(CM-E-0033)_연구개발_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 10:00:48</t>
+          <t>2026-08-18 10:26:49</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -3058,12 +3058,12 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>CM-0038 레이저길이 측정기</t>
+          <t>CM-0041 토크 드라이버</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0041 260306 - 토크드라이버(CM-E-0033)_연구개발.pdf</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3115,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>CM-0038_레이저길이 측정기_241004_개발실(241002BG14)_적합성.PDF</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -3177,14 +3177,14 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>CM-0038_레이저길이 측정기_241004_개발실(241002BG14).PDF</t>
+          <t>CM-0038_레이저길이 측정기_241004_개발실(241002BG14)_적합성.PDF</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:58:34</t>
+          <t>2026-08-18 10:00:48</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>CM-0037 1m 곧은자</t>
+          <t>CM-0038 레이저길이 측정기</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0038_레이저길이 측정기_241004_개발실(241002BG14).PDF</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>CM-0037_곧은 자 1M_250709_현장(25009308-1)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -3333,14 +3333,14 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>CM-0037_곧은 자 1M_250709_현장(25009308-1).pdf</t>
+          <t>CM-0037_곧은 자 1M_250709_현장(25009308-1)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:57:43</t>
+          <t>2026-08-18 09:58:34</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3370,12 +3370,12 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>CM-0036 30m 줄자</t>
+          <t>CM-0037 1m 곧은자</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0037_곧은 자 1M_250709_현장(25009308-1).pdf</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>CM-0036_30m 줄자_250709_현장(25003413-1)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -3489,14 +3489,14 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>CM-0036_30m 줄자_250709_현장(25003413-1).pdf</t>
+          <t>CM-0036_30m 줄자_250709_현장(25003413-1)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:56:34</t>
+          <t>2026-08-18 09:57:43</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3526,12 +3526,12 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>CM-0035 5.5m 줄자</t>
+          <t>CM-0036 30m 줄자</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3541,7 +3541,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0036_30m 줄자_250709_현장(25003413-1).pdf</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>CM-0035_5.5m 줄자_250709_현장(25009308-3)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -3645,14 +3645,14 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>CM-0035_5.5m 줄자_250709_현장(25009308-3).pdf</t>
+          <t>CM-0035_5.5m 줄자_250709_현장(25009308-3)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:55:12</t>
+          <t>2026-08-18 09:56:34</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3682,12 +3682,12 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>CM-0034 온·습도계</t>
+          <t>CM-0035 5.5m 줄자</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0035_5.5m 줄자_250709_현장(25009308-3).pdf</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0034_260714- 디지털온도계_AOA실_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -3801,14 +3801,14 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0034_260714- 디지털온도계_AOA실.pdf</t>
+          <t>관리번호 CM-0034_260714- 디지털온도계_AOA실_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:53:52</t>
+          <t>2026-08-18 09:55:12</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3838,12 +3838,12 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>CM-0033 CABLE&amp;HARNESS MULTI TESTER</t>
+          <t>CM-0034 온·습도계</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -3853,14 +3853,14 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0034_260714- 디지털온도계_AOA실.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:52:51</t>
+          <t>2026-08-18 09:53:52</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>CM-0032 Oscilloscope</t>
+          <t>CM-0033 CABLE&amp;HARNESS MULTI TESTER</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -3957,7 +3957,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0032_260526-Oscilloscope(RTM3004)_대전연구소_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -4009,14 +4009,14 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0032_260526-Oscilloscope(RTM3004)_대전연구소.pdf</t>
+          <t>관리번호 CM-0032_260526-Oscilloscope(RTM3004)_대전연구소_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:51:15</t>
+          <t>2026-08-18 09:52:51</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4046,12 +4046,12 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>CM-0031 AC Power Supply</t>
+          <t>CM-0032 Oscilloscope</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0032_260526-Oscilloscope(RTM3004)_대전연구소.pdf</t>
         </is>
       </c>
     </row>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0031_260202 - AC Power Supply_AOA실_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -4165,14 +4165,14 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0031_260202 - AC Power Supply_AOA실.pdf</t>
+          <t>관리번호 CM-0031_260202 - AC Power Supply_AOA실_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:50:13</t>
+          <t>2026-08-18 09:51:15</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4202,12 +4202,12 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>CM-0030 DC Power Supply</t>
+          <t>CM-0031 AC Power Supply</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0031_260202 - AC Power Supply_AOA실.pdf</t>
         </is>
       </c>
     </row>
@@ -4259,7 +4259,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0030_260527-Dc Power Supply(E36233A)_대전연구소_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -4321,14 +4321,14 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0030_260527-Dc Power Supply(E36233A)_대전연구소.pdf</t>
+          <t>관리번호 CM-0030_260527-Dc Power Supply(E36233A)_대전연구소_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:48:25</t>
+          <t>2026-08-18 09:50:13</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4358,12 +4358,12 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>CM-0022 광 측정기</t>
+          <t>CM-0030 DC Power Supply</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -4373,14 +4373,14 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0030_260527-Dc Power Supply(E36233A)_대전연구소.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:47:38</t>
+          <t>2026-08-18 09:48:25</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>CM-0029 StopWatch</t>
+          <t>CM-0022 광 측정기</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0029_260327 - 초시계_StopWatch-_AOA실_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -4529,14 +4529,14 @@
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0029_260327 - 초시계_StopWatch-_AOA실.pdf</t>
+          <t>관리번호 CM-0029_260327 - 초시계_StopWatch-_AOA실_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:45:50</t>
+          <t>2026-08-18 09:47:38</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4566,12 +4566,12 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>CM-0028 DC Power Supply</t>
+          <t>CM-0029 StopWatch</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0029_260327 - 초시계_StopWatch-_AOA실.pdf</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0028_260326 - DC POWER SUPPY(GPE-4323)_개발실_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -4685,14 +4685,14 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0028_260326 - DC POWER SUPPY(GPE-4323)_개발실.pdf</t>
+          <t>관리번호 CM-0028_260326 - DC POWER SUPPY(GPE-4323)_개발실_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:43:13</t>
+          <t>2026-08-18 09:45:50</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4722,12 +4722,12 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>CM-0027 Multimeter</t>
+          <t>CM-0028 DC Power Supply</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0028_260326 - DC POWER SUPPY(GPE-4323)_개발실.pdf</t>
         </is>
       </c>
     </row>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0027_260327 - DCIGITAK MULTIMETER(MY6006711)_AOA실_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -4841,14 +4841,14 @@
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0027_260327 - DCIGITAK MULTIMETER(MY6006711)_AOA실.pdf</t>
+          <t>관리번호 CM-0027_260327 - DCIGITAK MULTIMETER(MY6006711)_AOA실_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:41:32</t>
+          <t>2026-08-18 09:43:13</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4878,12 +4878,12 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>CM-0026 디지털 온습도계</t>
+          <t>CM-0027 Multimeter</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0027_260327 - DCIGITAK MULTIMETER(MY6006711)_AOA실.pdf</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>CM-0026_디지털 온습도계_251219_생산실1(25017233-2)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -4997,14 +4997,14 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>CM-0026_디지털 온습도계_251219_생산실1(25017233-2).pdf</t>
+          <t>CM-0026_디지털 온습도계_251219_생산실1(25017233-2)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:40:35</t>
+          <t>2026-08-18 09:41:32</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -5034,12 +5034,12 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>CM-0025 디지털 온습도계</t>
+          <t>CM-0026 디지털 온습도계</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0026_디지털 온습도계_251219_생산실1(25017233-2).pdf</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>CM-0025_디지털 온습도계_251219_자재실1(25017233-3)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -5153,14 +5153,14 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>CM-0025_디지털 온습도계_251219_자재실1(25017233-3).pdf</t>
+          <t>CM-0025_디지털 온습도계_251219_자재실1(25017233-3)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:39:41</t>
+          <t>2026-08-18 09:40:35</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5190,12 +5190,12 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>CM-0024 디지털 온습도계</t>
+          <t>CM-0025 디지털 온습도계</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0025_디지털 온습도계_251219_자재실1(25017233-3).pdf</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>CM-0024_디지털 온습도계_251219_AOA생산실(25017233-1)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -5309,14 +5309,14 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>CM-0024_디지털 온습도계_251219_AOA생산실(25017233-1).pdf</t>
+          <t>CM-0024_디지털 온습도계_251219_AOA생산실(25017233-1)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:38:50</t>
+          <t>2026-08-18 09:39:41</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -5346,12 +5346,12 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>CM-0023 디지털 온습도계</t>
+          <t>CM-0024 디지털 온습도계</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -5361,7 +5361,7 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0024_디지털 온습도계_251219_AOA생산실(25017233-1).pdf</t>
         </is>
       </c>
     </row>
@@ -5403,7 +5403,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
@@ -5413,7 +5413,7 @@
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>CM-0023_디지털 온습도계_251219_자재실2(25017233-4)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -5465,14 +5465,14 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>CM-0023_디지털 온습도계_251219_자재실2(25017233-4).pdf</t>
+          <t>CM-0023_디지털 온습도계_251219_자재실2(25017233-4)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:37:33</t>
+          <t>2026-08-18 09:38:50</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5502,12 +5502,12 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>CM-0021 휘도계</t>
+          <t>CM-0023 디지털 온습도계</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0023_디지털 온습도계_251219_자재실2(25017233-4).pdf</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>CM-0021_휘도계_251016_생산실(251015EJ40)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -5621,14 +5621,14 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>CM-0021_휘도계_251016_생산실(251015EJ40).pdf</t>
+          <t>CM-0021_휘도계_251016_생산실(251015EJ40)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:36:38</t>
+          <t>2026-08-18 09:37:33</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -5658,12 +5658,12 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>CM-0020 전기식 지시저울</t>
+          <t>CM-0021 휘도계</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0021_휘도계_251016_생산실(251015EJ40).pdf</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5715,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
@@ -5725,7 +5725,7 @@
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>CM-0020_전기식 지시저울_251002_현장(25013530-6)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -5777,14 +5777,14 @@
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>CM-0020_전기식 지시저울_251002_현장(25013530-6).pdf</t>
+          <t>CM-0020_전기식 지시저울_251002_현장(25013530-6)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:35:39</t>
+          <t>2026-08-18 09:36:38</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5814,12 +5814,12 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>CM-0019 Multimeter</t>
+          <t>CM-0020 전기식 지시저울</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0020_전기식 지시저울_251002_현장(25013530-6).pdf</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
-          <t>CM-0019_INSULATION MULTIMETER_251002_현장(25013530-4)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -5933,14 +5933,14 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>CM-0019_INSULATION MULTIMETER_251002_현장(25013530-4).pdf</t>
+          <t>CM-0019_INSULATION MULTIMETER_251002_현장(25013530-4)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:34:03</t>
+          <t>2026-08-18 09:35:39</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -5970,12 +5970,12 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>CM-0018 DC Power Supply</t>
+          <t>CM-0019 Multimeter</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
@@ -5985,7 +5985,7 @@
       </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0019_INSULATION MULTIMETER_251002_현장(25013530-4).pdf</t>
         </is>
       </c>
     </row>
@@ -6027,7 +6027,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
@@ -6037,7 +6037,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>CM-0018_DC Power Supply_251002_AOA생산실(25013530-7)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -6089,14 +6089,14 @@
       </c>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>CM-0018_DC Power Supply_251002_AOA생산실(25013530-7).pdf</t>
+          <t>CM-0018_DC Power Supply_251002_AOA생산실(25013530-7)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:31:55</t>
+          <t>2026-08-18 09:34:03</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -6126,12 +6126,12 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>CM-0017 mΩ HiTESTER</t>
+          <t>CM-0018 DC Power Supply</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0018_DC Power Supply_251002_AOA생산실(25013530-7).pdf</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -6193,7 +6193,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0017_260805_ mΩ HiTESTER_현장_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -6245,14 +6245,14 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>관리번호 CM-0017_260805_ mΩ HiTESTER_현장 .pdf</t>
+          <t>관리번호 CM-0017_260805_ mΩ HiTESTER_현장_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:29:41</t>
+          <t>2026-08-18 09:31:55</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -6282,12 +6282,12 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>CM-0016 광조도계</t>
+          <t>CM-0017 mΩ HiTESTER</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>관리번호 CM-0017_260805_ mΩ HiTESTER_현장 .pdf</t>
         </is>
       </c>
     </row>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr">
@@ -6349,7 +6349,7 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>CM-0016_광조도계_250903_개발실(25021404-1)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -6401,14 +6401,14 @@
       </c>
       <c r="J121" s="2" t="inlineStr">
         <is>
-          <t>CM-0016_광조도계_250903_개발실(25021404-1).pdf</t>
+          <t>CM-0016_광조도계_250903_개발실(25021404-1)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:28:42</t>
+          <t>2026-08-18 09:29:41</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -6438,12 +6438,12 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>CM-0015 휘도계</t>
+          <t>CM-0016 광조도계</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0016_광조도계_250903_개발실(25021404-1).pdf</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr">
@@ -6505,7 +6505,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>CM-0015_휘도계(LUMINANCE COLORI METER)_250909_생산실(250903EM64)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -6557,14 +6557,14 @@
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>CM-0015_휘도계(LUMINANCE COLORI METER)_250909_생산실(250903EM64).pdf</t>
+          <t>CM-0015_휘도계(LUMINANCE COLORI METER)_250909_생산실(250903EM64)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:27:44</t>
+          <t>2026-08-18 09:28:42</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -6594,12 +6594,12 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>CM-0014 듀얼축 각도기</t>
+          <t>CM-0015 휘도계</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0015_휘도계(LUMINANCE COLORI METER)_250909_생산실(250903EM64).pdf</t>
         </is>
       </c>
     </row>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
@@ -6661,7 +6661,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>CM-0014_각도 정규(듀얼축 각도기)_250901_개발실(25011747-11)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -6713,14 +6713,14 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>CM-0014_각도 정규(듀얼축 각도기)_250901_개발실(25011747-11).pdf</t>
+          <t>CM-0014_각도 정규(듀얼축 각도기)_250901_개발실(25011747-11)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:26:09</t>
+          <t>2026-08-18 09:27:44</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -6750,12 +6750,12 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>CM-0013 버니어켈리퍼스</t>
+          <t>CM-0014 듀얼축 각도기</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr">
@@ -6765,7 +6765,7 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0014_각도 정규(듀얼축 각도기)_250901_개발실(25011747-11).pdf</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I129" s="2" t="inlineStr">
@@ -6817,7 +6817,7 @@
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>CM-0013_내외측캘리퍼(버니어캐리퍼스)_251013_개발실(25013530-2)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -6869,14 +6869,14 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>CM-0013_내외측캘리퍼(버니어캐리퍼스)_251013_개발실(25013530-2).pdf</t>
+          <t>CM-0013_내외측캘리퍼(버니어캐리퍼스)_251013_개발실(25013530-2)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:25:11</t>
+          <t>2026-08-18 09:26:09</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -6906,12 +6906,12 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>CM-0012 버니어켈리퍼스</t>
+          <t>CM-0013 버니어켈리퍼스</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I131" s="2" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0013_내외측캘리퍼(버니어캐리퍼스)_251013_개발실(25013530-2).pdf</t>
         </is>
       </c>
     </row>
@@ -6963,7 +6963,7 @@
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I132" s="2" t="inlineStr">
@@ -6973,7 +6973,7 @@
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>CM-0012_내외측캘리퍼(버니어캐리퍼스)_250901_개발실(25011747-8)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -7025,14 +7025,14 @@
       </c>
       <c r="J133" s="2" t="inlineStr">
         <is>
-          <t>CM-0012_내외측캘리퍼(버니어캐리퍼스)_250901_개발실(25011747-8).pdf</t>
+          <t>CM-0012_내외측캘리퍼(버니어캐리퍼스)_250901_개발실(25011747-8)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:24:13</t>
+          <t>2026-08-18 09:25:11</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -7062,12 +7062,12 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>CM-0011 버니어켈리퍼스</t>
+          <t>CM-0012 버니어켈리퍼스</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I134" s="2" t="inlineStr">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0012_내외측캘리퍼(버니어캐리퍼스)_250901_개발실(25011747-8).pdf</t>
         </is>
       </c>
     </row>
@@ -7119,7 +7119,7 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I135" s="2" t="inlineStr">
@@ -7129,7 +7129,7 @@
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>CM-0011_내외측캘리퍼(버니어캐리퍼스)_250901_개발실(25011747-9)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -7181,14 +7181,14 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>CM-0011_내외측캘리퍼(버니어캐리퍼스)_250901_개발실(25011747-9).pdf</t>
+          <t>CM-0011_내외측캘리퍼(버니어캐리퍼스)_250901_개발실(25011747-9)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:23:00</t>
+          <t>2026-08-18 09:24:13</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -7218,12 +7218,12 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>CM-0010 온도측정기</t>
+          <t>CM-0011 버니어켈리퍼스</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I137" s="2" t="inlineStr">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0011_내외측캘리퍼(버니어캐리퍼스)_250901_개발실(25011747-9).pdf</t>
         </is>
       </c>
     </row>
@@ -7275,7 +7275,7 @@
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I138" s="2" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>CM-0010_복사온도계(온도측정기)_250912_개발실(25012472-1)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -7337,14 +7337,14 @@
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t>CM-0010_복사온도계(온도측정기)_250912_개발실(25012472-1).pdf</t>
+          <t>CM-0010_복사온도계(온도측정기)_250912_개발실(25012472-1)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:20:42</t>
+          <t>2026-08-18 09:23:00</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -7374,12 +7374,12 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>CM-0008 Milliohm Meter</t>
+          <t>CM-0010 온도측정기</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I140" s="2" t="inlineStr">
@@ -7389,7 +7389,7 @@
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0010_복사온도계(온도측정기)_250912_개발실(25012472-1).pdf</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I141" s="2" t="inlineStr">
@@ -7441,7 +7441,7 @@
       </c>
       <c r="J141" s="2" t="inlineStr">
         <is>
-          <t>CM-0008_Milliohm Meter_250829_AOA생산실_(25011747-3)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -7493,14 +7493,14 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>CM-0008_Milliohm Meter_250829_AOA생산실_(25011747-3).pdf</t>
+          <t>CM-0008_Milliohm Meter_250829_AOA생산실_(25011747-3)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:19:48</t>
+          <t>2026-08-18 09:20:42</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -7530,12 +7530,12 @@
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>CM-0007 TRUE RMS Multimeter</t>
+          <t>CM-0008 Milliohm Meter</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I143" s="2" t="inlineStr">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0008_Milliohm Meter_250829_AOA생산실_(25011747-3).pdf</t>
         </is>
       </c>
     </row>
@@ -7587,7 +7587,7 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr">
@@ -7597,7 +7597,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>CM-0007_TRUE RMS Multimeter_250829_개발실(25011747-4)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -7649,14 +7649,14 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>CM-0007_TRUE RMS Multimeter_250829_개발실(25011747-4).pdf</t>
+          <t>CM-0007_TRUE RMS Multimeter_250829_개발실(25011747-4)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:18:31</t>
+          <t>2026-08-18 09:19:48</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -7686,12 +7686,12 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>CM-0006 TRUE RMS Multimeter</t>
+          <t>CM-0007 TRUE RMS Multimeter</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0007_TRUE RMS Multimeter_250829_개발실(25011747-4).pdf</t>
         </is>
       </c>
     </row>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I147" s="2" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="J147" s="2" t="inlineStr">
         <is>
-          <t>CM-0006_TRUE RMS Multimeter_250829_ 개발실(25011747-5)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -7805,14 +7805,14 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>CM-0006_TRUE RMS Multimeter_250829_ 개발실(25011747-5).pdf</t>
+          <t>CM-0006_TRUE RMS Multimeter_250829_ 개발실(25011747-5)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:17:16</t>
+          <t>2026-08-18 09:18:31</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -7837,34 +7837,34 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>수정</t>
+          <t>등록</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>CM-0005 온·습도계</t>
+          <t>CM-0006 TRUE RMS Multimeter</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>계측기명</t>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>온습도계</t>
+          <t/>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
         <is>
-          <t>온·습도계</t>
+          <t>CM-0006_TRUE RMS Multimeter_250829_ 개발실(25011747-5).pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:17:00</t>
+          <t>2026-08-18 09:17:16</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -7889,27 +7889,27 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>등록</t>
+          <t>수정</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>CM-0005 온습도계</t>
+          <t>CM-0005 온·습도계</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>계측기명</t>
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>온습도계</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>온·습도계</t>
         </is>
       </c>
     </row>
@@ -7951,7 +7951,7 @@
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I151" s="2" t="inlineStr">
@@ -7961,7 +7961,7 @@
       </c>
       <c r="J151" s="2" t="inlineStr">
         <is>
-          <t>CM-0005_온습도계_251014_현장(25013530-3)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -8013,14 +8013,14 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>CM-0005_온습도계_251014_현장(25013530-3).pdf</t>
+          <t>CM-0005_온습도계_251014_현장(25013530-3)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:15:36</t>
+          <t>2026-08-18 09:17:00</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -8050,12 +8050,12 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>CM-0004 온·습도계</t>
+          <t>CM-0005 온습도계</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
@@ -8065,7 +8065,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0005_온습도계_251014_현장(25013530-3).pdf</t>
         </is>
       </c>
     </row>
@@ -8107,7 +8107,7 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>CM-0004_온습도계_250829_자재실(25011747-7)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -8169,14 +8169,14 @@
       </c>
       <c r="J155" s="2" t="inlineStr">
         <is>
-          <t>CM-0004_온습도계_250829_자재실(25011747-7).pdf</t>
+          <t>CM-0004_온습도계_250829_자재실(25011747-7)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:13:28</t>
+          <t>2026-08-18 09:15:36</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -8206,12 +8206,12 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>CM-0003 Oscilloscope</t>
+          <t>CM-0004 온·습도계</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I156" s="2" t="inlineStr">
@@ -8221,7 +8221,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0004_온습도계_250829_자재실(25011747-7).pdf</t>
         </is>
       </c>
     </row>
@@ -8263,7 +8263,7 @@
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I157" s="2" t="inlineStr">
@@ -8273,7 +8273,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>CM-0003_Oscilloscope_250919_현장(WO-01196944)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -8325,14 +8325,14 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>CM-0003_Oscilloscope_250919_현장(WO-01196944).pdf</t>
+          <t>CM-0003_Oscilloscope_250919_현장(WO-01196944)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:09:52</t>
+          <t>2026-08-18 09:13:28</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -8362,12 +8362,12 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>CM-0002 DC Power Supply</t>
+          <t>CM-0003 Oscilloscope</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I159" s="2" t="inlineStr">
@@ -8377,7 +8377,7 @@
       </c>
       <c r="J159" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0003_Oscilloscope_250919_현장(WO-01196944).pdf</t>
         </is>
       </c>
     </row>
@@ -8419,7 +8419,7 @@
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>첨부 추가</t>
+          <t/>
         </is>
       </c>
       <c r="I160" s="2" t="inlineStr">
@@ -8429,7 +8429,7 @@
       </c>
       <c r="J160" s="2" t="inlineStr">
         <is>
-          <t>CM-0002_DC Power Supply_250829_개발실(25011747-2)_적합성.pdf</t>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -8481,14 +8481,14 @@
       </c>
       <c r="J161" s="2" t="inlineStr">
         <is>
-          <t>CM-0002_DC Power Supply_250829_개발실(25011747-2).pdf</t>
+          <t>CM-0002_DC Power Supply_250829_개발실(25011747-2)_적합성.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:07:26</t>
+          <t>2026-08-18 09:09:52</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -8518,12 +8518,12 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>CM-0001 DC Power Supply</t>
+          <t>CM-0002 DC Power Supply</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>첨부 추가</t>
         </is>
       </c>
       <c r="I162" s="2" t="inlineStr">
@@ -8533,14 +8533,14 @@
       </c>
       <c r="J162" s="2" t="inlineStr">
         <is>
-          <t>계측기 등록</t>
+          <t>CM-0002_DC Power Supply_250829_개발실(25011747-2).pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:01:07</t>
+          <t>2026-08-18 09:07:26</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -8565,27 +8565,27 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>수정</t>
+          <t>등록</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>CM-0009 적외선 온도계</t>
+          <t>CM-0001 DC Power Supply</t>
         </is>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
-          <t>사용 부서</t>
+          <t/>
         </is>
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>현장</t>
+          <t/>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>계측기 등록</t>
         </is>
       </c>
     </row>
@@ -8627,24 +8627,24 @@
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>설치 위치</t>
+          <t>사용 부서</t>
         </is>
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>현장</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
         <is>
-          <t>현장</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 08:55:35</t>
+          <t>2026-08-18 09:01:07</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
@@ -8679,7 +8679,7 @@
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>사용 부서</t>
+          <t>설치 위치</t>
         </is>
       </c>
       <c r="I165" s="2" t="inlineStr">
@@ -8696,50 +8696,102 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
+          <t>2026-08-18 08:55:35</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>주식회사 카프마이크로</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>박준영</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>jypark@caphmicro.com</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>계측기 통합 대장</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>수정</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>CM-0009 적외선 온도계</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>사용 부서</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
           <t>2026-08-18 08:34:49</t>
         </is>
       </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>주식회사 카프마이크로</t>
-        </is>
-      </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>박준영</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr">
-        <is>
-          <t>jypark@caphmicro.com</t>
-        </is>
-      </c>
-      <c r="E166" s="2" t="inlineStr">
-        <is>
-          <t>계측기 통합 대장</t>
-        </is>
-      </c>
-      <c r="F166" s="2" t="inlineStr">
-        <is>
-          <t>등록</t>
-        </is>
-      </c>
-      <c r="G166" s="2" t="inlineStr">
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>주식회사 카프마이크로</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>박준영</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>jypark@caphmicro.com</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>계측기 통합 대장</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>등록</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
         <is>
           <t>CM-0009 적외선 온도계</t>
         </is>
       </c>
-      <c r="H166" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I166" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J166" s="2" t="inlineStr">
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr">
         <is>
           <t>계측기 등록</t>
         </is>

</xml_diff>